<commit_message>
Add milk, cream and permeate transfers between sites
- New optional input sheets Transfer_Types (kg/kL composition range per
  component) and Transfer_Routes (cost per kL, weekly limit); older
  workbooks without them still load
- Transfers move components between factories' MILK pools; whole-milk
  transfers count toward receiving intake and move the lactoferrin limit
- Transfers results sheet, P&L line and console summary
- Tests for composition/limits and backward compatibility; design doc,
  sample inputs and results updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012yktA7hQJGuh9yaJQaiyLA
</commit_message>
<xml_diff>
--- a/data/sample_inputs.xlsx
+++ b/data/sample_inputs.xlsx
@@ -23,6 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant_Hours" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spot" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer_Types" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer_Routes" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,10 +434,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -632,16 +634,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Transfer_Types</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>What can be moved between sites (milk, cream, permeate) and its kg/kL composition range</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Transfer_Routes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Allowed site-to-site transfers, cost $/kL and weekly limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>All data in this workbook is made up for demonstration purposes.</t>
         </is>
@@ -25285,6 +25311,741 @@
       </c>
       <c r="C53" t="n">
         <v>733</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>transfer_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>source_stream</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dest_stream</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>whole_milk</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fat_min_kg_per_kL</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fat_max_kg_per_kL</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>protein_min_kg_per_kL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>protein_max_kg_per_kL</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>la_min_kg_per_kL</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>la_max_kg_per_kL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Whole milk (standardised within a normal milk range)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G2" t="n">
+        <v>47</v>
+      </c>
+      <c r="H2" t="n">
+        <v>31</v>
+      </c>
+      <c r="I2" t="n">
+        <v>37</v>
+      </c>
+      <c r="J2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K2" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cream ~40% fat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>380</v>
+      </c>
+      <c r="G3" t="n">
+        <v>420</v>
+      </c>
+      <c r="H3" t="n">
+        <v>18</v>
+      </c>
+      <c r="I3" t="n">
+        <v>22</v>
+      </c>
+      <c r="J3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K3" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UF permeate, RO-concentrated to ~18% solids</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>170</v>
+      </c>
+      <c r="K4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>transfer_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>from_factory</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>to_factory</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>distance_km</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cost_per_kL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>max_kL_per_week</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>310</v>
+      </c>
+      <c r="E2" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>310</v>
+      </c>
+      <c r="E3" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>540</v>
+      </c>
+      <c r="E4" t="n">
+        <v>81</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>540</v>
+      </c>
+      <c r="E5" t="n">
+        <v>81</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>820</v>
+      </c>
+      <c r="E6" t="n">
+        <v>123</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MILK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>820</v>
+      </c>
+      <c r="E7" t="n">
+        <v>123</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>310</v>
+      </c>
+      <c r="E8" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>310</v>
+      </c>
+      <c r="E9" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>540</v>
+      </c>
+      <c r="E10" t="n">
+        <v>81</v>
+      </c>
+      <c r="F10" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>540</v>
+      </c>
+      <c r="E11" t="n">
+        <v>81</v>
+      </c>
+      <c r="F11" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>820</v>
+      </c>
+      <c r="E12" t="n">
+        <v>123</v>
+      </c>
+      <c r="F12" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CREAM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>820</v>
+      </c>
+      <c r="E13" t="n">
+        <v>123</v>
+      </c>
+      <c r="F13" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>310</v>
+      </c>
+      <c r="E14" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>310</v>
+      </c>
+      <c r="E15" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>540</v>
+      </c>
+      <c r="E16" t="n">
+        <v>81</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>540</v>
+      </c>
+      <c r="E17" t="n">
+        <v>81</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>820</v>
+      </c>
+      <c r="E18" t="n">
+        <v>123</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PERMEATE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CYG</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>820</v>
+      </c>
+      <c r="E19" t="n">
+        <v>123</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Set confirmed transfer specs: cream 40% fat, permeate 18% solids
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012yktA7hQJGuh9yaJQaiyLA
</commit_message>
<xml_diff>
--- a/data/sample_inputs.xlsx
+++ b/data/sample_inputs.xlsx
@@ -25328,7 +25328,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="73" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -25448,7 +25448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cream ~40% fat</t>
+          <t>Cream 40% fat (~396 kg fat/kL at 0.99 kg/L)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -25465,10 +25465,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="G3" t="n">
-        <v>420</v>
+        <v>400</v>
       </c>
       <c r="H3" t="n">
         <v>18</v>
@@ -25491,7 +25491,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>UF permeate, RO-concentrated to ~18% solids</t>
+          <t>UF permeate concentrated to 18% solids (~193 kg solids/kL at 1.07 kg/L)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -25520,7 +25520,7 @@
         <v>8</v>
       </c>
       <c r="J4" t="n">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="K4" t="n">
         <v>190</v>

</xml_diff>